<commit_message>
update thesis v5 + include ML docs
</commit_message>
<xml_diff>
--- a/Docs/ARIMA_Metrics_Summary_v1.1.xlsx
+++ b/Docs/ARIMA_Metrics_Summary_v1.1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frank\Downloads\PyUtilities\Stoch-Mort-With-ML\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAB5C219-05B6-4BF2-9B69-EB2EA3126A6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E04C0E8-32BE-473D-8FA9-97C6508B19F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{2D876342-0684-4DCF-83A6-6F1E2B654471}"/>
   </bookViews>
@@ -811,7 +811,7 @@
     <col min="9" max="9" width="15.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17.5703125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.5703125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="8.7109375" bestFit="1" customWidth="1"/>

</xml_diff>